<commit_message>
CHANGES DONE ON 26TH AUGUST
</commit_message>
<xml_diff>
--- a/12603864.xlsx
+++ b/12603864.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP 776\12603864\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1E25A276-15EE-4A4F-A668-1D9BE6F8C706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{547D2886-00AA-4B0A-833C-C062A67016CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -218,6 +218,15 @@
   </si>
   <si>
     <t>COULD HAVE DONE MORE, BIT DISTRACTED REGARDING CERTAIN THINGS</t>
+  </si>
+  <si>
+    <t>SATISFACTORY</t>
+  </si>
+  <si>
+    <t>HIGH</t>
+  </si>
+  <si>
+    <t>GREAT DAY</t>
   </si>
 </sst>
 </file>
@@ -1089,26 +1098,50 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="13"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="15" t="str">
+      <c r="A8" s="13">
+        <v>46258</v>
+      </c>
+      <c r="B8" s="14">
+        <v>400</v>
+      </c>
+      <c r="C8" s="14">
+        <v>40</v>
+      </c>
+      <c r="D8" s="14">
+        <v>200</v>
+      </c>
+      <c r="E8" s="14">
+        <v>40</v>
+      </c>
+      <c r="F8" s="14">
+        <v>0</v>
+      </c>
+      <c r="G8" s="14">
+        <v>0</v>
+      </c>
+      <c r="H8" s="14">
+        <v>480</v>
+      </c>
+      <c r="I8" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J8" s="15" t="str">
+        <v>1160</v>
+      </c>
+      <c r="J8" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="17"/>
+        <v>280</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N8" s="17" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="13"/>

</xml_diff>

<commit_message>
Updated on 27th August
</commit_message>
<xml_diff>
--- a/12603864.xlsx
+++ b/12603864.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP 776\12603864\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{547D2886-00AA-4B0A-833C-C062A67016CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38DDB018-95ED-4E4C-8FD2-BEC4E3F6A3C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="66">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -227,6 +227,12 @@
   </si>
   <si>
     <t>GREAT DAY</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>JUST A REGULAR LAZY DAY</t>
   </si>
 </sst>
 </file>
@@ -1144,26 +1150,50 @@
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15" t="str">
+      <c r="A9" s="13">
+        <v>46261</v>
+      </c>
+      <c r="B9" s="14">
+        <v>420</v>
+      </c>
+      <c r="C9" s="14">
+        <v>40</v>
+      </c>
+      <c r="D9" s="14">
+        <v>0</v>
+      </c>
+      <c r="E9" s="14">
+        <v>0</v>
+      </c>
+      <c r="F9" s="14">
+        <v>420</v>
+      </c>
+      <c r="G9" s="14">
+        <v>7</v>
+      </c>
+      <c r="H9" s="14">
+        <v>90</v>
+      </c>
+      <c r="I9" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J9" s="15" t="str">
+        <v>970</v>
+      </c>
+      <c r="J9" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="17"/>
+        <v>470</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="13"/>

</xml_diff>

<commit_message>
Updated on 28th august
</commit_message>
<xml_diff>
--- a/12603864.xlsx
+++ b/12603864.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP 776\12603864\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38DDB018-95ED-4E4C-8FD2-BEC4E3F6A3C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC6ABF34-5C74-4603-B3A8-51146262C88F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -233,6 +233,12 @@
   </si>
   <si>
     <t>JUST A REGULAR LAZY DAY</t>
+  </si>
+  <si>
+    <t>GOOD</t>
+  </si>
+  <si>
+    <t>HAD A PRODUCTIVE DAY TODAY , BETTER THAN REST OF THE DAYS</t>
   </si>
 </sst>
 </file>
@@ -1195,27 +1201,51 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="15" t="str">
+    <row r="10" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="13">
+        <v>46262</v>
+      </c>
+      <c r="B10" s="14">
+        <v>450</v>
+      </c>
+      <c r="C10" s="14">
+        <v>30</v>
+      </c>
+      <c r="D10" s="14">
+        <v>330</v>
+      </c>
+      <c r="E10" s="14">
+        <v>40</v>
+      </c>
+      <c r="F10" s="14">
+        <v>240</v>
+      </c>
+      <c r="G10" s="14">
+        <v>4</v>
+      </c>
+      <c r="H10" s="14">
+        <v>60</v>
+      </c>
+      <c r="I10" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J10" s="15" t="str">
+        <v>1150</v>
+      </c>
+      <c r="J10" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
-      <c r="N10" s="17"/>
+        <v>290</v>
+      </c>
+      <c r="K10" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L10" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N10" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="13"/>

</xml_diff>

<commit_message>
Updated on 30th August 2026
</commit_message>
<xml_diff>
--- a/12603864.xlsx
+++ b/12603864.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP 776\12603864\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC6ABF34-5C74-4603-B3A8-51146262C88F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{672C8B41-B5D7-4B8D-8DC5-4C215DA37860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="71">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -239,6 +239,15 @@
   </si>
   <si>
     <t>HAD A PRODUCTIVE DAY TODAY , BETTER THAN REST OF THE DAYS</t>
+  </si>
+  <si>
+    <t>WORST</t>
+  </si>
+  <si>
+    <t>NOT SATISFACTORY</t>
+  </si>
+  <si>
+    <t>JUST A REGULAR DAY WITH SOME BAD MOMENTS</t>
   </si>
 </sst>
 </file>
@@ -1247,27 +1256,51 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="13"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="15" t="str">
+    <row r="11" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="13">
+        <v>46263</v>
+      </c>
+      <c r="B11" s="14">
+        <v>480</v>
+      </c>
+      <c r="C11" s="14">
+        <v>40</v>
+      </c>
+      <c r="D11" s="14">
+        <v>420</v>
+      </c>
+      <c r="E11" s="14">
+        <v>60</v>
+      </c>
+      <c r="F11" s="14">
+        <v>0</v>
+      </c>
+      <c r="G11" s="14">
+        <v>0</v>
+      </c>
+      <c r="H11" s="14">
+        <v>90</v>
+      </c>
+      <c r="I11" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="15" t="str">
+        <v>1090</v>
+      </c>
+      <c r="J11" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="17"/>
+        <v>350</v>
+      </c>
+      <c r="K11" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>

</xml_diff>

<commit_message>
Updated on 31st August 2026
</commit_message>
<xml_diff>
--- a/12603864.xlsx
+++ b/12603864.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP 776\12603864\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{672C8B41-B5D7-4B8D-8DC5-4C215DA37860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E268DA8-9168-4EED-B6B2-AD83B082DBA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="73">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -248,6 +248,12 @@
   </si>
   <si>
     <t>JUST A REGULAR DAY WITH SOME BAD MOMENTS</t>
+  </si>
+  <si>
+    <t>NOT GOOD</t>
+  </si>
+  <si>
+    <t>WASTED A LOT OF TIME</t>
   </si>
 </sst>
 </file>
@@ -1302,27 +1308,51 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+    <row r="12" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="13">
+        <v>46264</v>
+      </c>
+      <c r="B12" s="14">
+        <v>480</v>
+      </c>
+      <c r="C12" s="14">
+        <v>40</v>
+      </c>
+      <c r="D12" s="14">
+        <v>360</v>
+      </c>
+      <c r="E12" s="14">
+        <v>30</v>
+      </c>
+      <c r="F12" s="14">
+        <v>0</v>
+      </c>
+      <c r="G12" s="14">
+        <v>0</v>
+      </c>
+      <c r="H12" s="14">
+        <v>60</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>970</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="17"/>
+        <v>470</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="13"/>

</xml_diff>

<commit_message>
Updated on 3rd September 2026
</commit_message>
<xml_diff>
--- a/12603864.xlsx
+++ b/12603864.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP 776\12603864\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E268DA8-9168-4EED-B6B2-AD83B082DBA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F6503C-D53B-4AFC-A5AD-F9A1921BF9CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="77">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -254,6 +254,18 @@
   </si>
   <si>
     <t>WASTED A LOT OF TIME</t>
+  </si>
+  <si>
+    <t>NOT DONE MUCH</t>
+  </si>
+  <si>
+    <t>VERY LOW</t>
+  </si>
+  <si>
+    <t>JUST SLEPT A LOT AND WASTED TIME</t>
+  </si>
+  <si>
+    <t>WASTED WHOLE DAY</t>
   </si>
 </sst>
 </file>
@@ -1354,71 +1366,143 @@
         <v>72</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15" t="str">
+    <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="13">
+        <v>46265</v>
+      </c>
+      <c r="B13" s="14">
+        <v>480</v>
+      </c>
+      <c r="C13" s="14">
+        <v>30</v>
+      </c>
+      <c r="D13" s="14">
+        <v>300</v>
+      </c>
+      <c r="E13" s="14">
+        <v>60</v>
+      </c>
+      <c r="F13" s="14">
+        <v>300</v>
+      </c>
+      <c r="G13" s="14">
+        <v>6</v>
+      </c>
+      <c r="H13" s="14">
+        <v>60</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
+        <v>1230</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="17"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+        <v>210</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="13">
+        <v>46266</v>
+      </c>
+      <c r="B14" s="14">
+        <v>540</v>
+      </c>
+      <c r="C14" s="14">
+        <v>0</v>
+      </c>
+      <c r="D14" s="14">
+        <v>0</v>
+      </c>
+      <c r="E14" s="14">
+        <v>0</v>
+      </c>
+      <c r="F14" s="14">
+        <v>350</v>
+      </c>
+      <c r="G14" s="14">
+        <v>7</v>
+      </c>
+      <c r="H14" s="14">
+        <v>90</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>980</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="17"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="13"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="str">
+        <v>460</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="13">
+        <v>46267</v>
+      </c>
+      <c r="B15" s="14">
+        <v>420</v>
+      </c>
+      <c r="C15" s="14">
+        <v>0</v>
+      </c>
+      <c r="D15" s="14">
+        <v>120</v>
+      </c>
+      <c r="E15" s="14">
+        <v>0</v>
+      </c>
+      <c r="F15" s="14">
+        <v>350</v>
+      </c>
+      <c r="G15" s="14">
+        <v>7</v>
+      </c>
+      <c r="H15" s="14">
+        <v>180</v>
+      </c>
+      <c r="I15" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="15" t="str">
+        <v>1070</v>
+      </c>
+      <c r="J15" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
-      <c r="N15" s="17"/>
+        <v>370</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="N15" s="17" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="13"/>

</xml_diff>

<commit_message>
Updated on 7th September 2026
</commit_message>
<xml_diff>
--- a/12603864.xlsx
+++ b/12603864.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP 776\12603864\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F6503C-D53B-4AFC-A5AD-F9A1921BF9CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D8E014D-5BA6-4DB5-A0F7-2A57A1FB962D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="80">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -266,6 +266,15 @@
   </si>
   <si>
     <t>WASTED WHOLE DAY</t>
+  </si>
+  <si>
+    <t>DIDNT WENT GOOD, DID WHAT I DIDN’T WANTED TO</t>
+  </si>
+  <si>
+    <t>IT WAS GOOD, NOT PRODUCTIVE THOUGH</t>
+  </si>
+  <si>
+    <t>WENT REALLY GOOD</t>
   </si>
 </sst>
 </file>
@@ -1504,115 +1513,235 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="str">
+    <row r="16" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="13">
+        <v>46268</v>
+      </c>
+      <c r="B16" s="14">
+        <v>420</v>
+      </c>
+      <c r="C16" s="14">
+        <v>60</v>
+      </c>
+      <c r="D16" s="14">
+        <v>300</v>
+      </c>
+      <c r="E16" s="14">
+        <v>60</v>
+      </c>
+      <c r="F16" s="14">
+        <v>250</v>
+      </c>
+      <c r="G16" s="14">
+        <v>5</v>
+      </c>
+      <c r="H16" s="14">
+        <v>60</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
+        <v>1150</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="17"/>
+        <v>290</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N16" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15" t="str">
+      <c r="A17" s="13">
+        <v>46269</v>
+      </c>
+      <c r="B17" s="14">
+        <v>420</v>
+      </c>
+      <c r="C17" s="14">
+        <v>60</v>
+      </c>
+      <c r="D17" s="14">
+        <v>180</v>
+      </c>
+      <c r="E17" s="14">
+        <v>40</v>
+      </c>
+      <c r="F17" s="14">
+        <v>250</v>
+      </c>
+      <c r="G17" s="14">
+        <v>5</v>
+      </c>
+      <c r="H17" s="14">
+        <v>60</v>
+      </c>
+      <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="15" t="str">
+        <v>1010</v>
+      </c>
+      <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
-      <c r="N17" s="17"/>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+        <v>430</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="13">
+        <v>46270</v>
+      </c>
+      <c r="B18" s="14">
+        <v>420</v>
+      </c>
+      <c r="C18" s="14">
+        <v>60</v>
+      </c>
+      <c r="D18" s="14">
+        <v>360</v>
+      </c>
+      <c r="E18" s="14">
+        <v>50</v>
+      </c>
+      <c r="F18" s="14">
+        <v>0</v>
+      </c>
+      <c r="G18" s="14">
+        <v>0</v>
+      </c>
+      <c r="H18" s="14">
+        <v>120</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>1010</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="17"/>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+        <v>430</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="13">
+        <v>46271</v>
+      </c>
+      <c r="B19" s="14">
+        <v>420</v>
+      </c>
+      <c r="C19" s="14">
+        <v>60</v>
+      </c>
+      <c r="D19" s="14">
+        <v>240</v>
+      </c>
+      <c r="E19" s="14">
+        <v>50</v>
+      </c>
+      <c r="F19" s="14">
+        <v>0</v>
+      </c>
+      <c r="G19" s="14">
+        <v>0</v>
+      </c>
+      <c r="H19" s="14">
+        <v>120</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>890</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="17"/>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+        <v>550</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="13">
+        <v>46272</v>
+      </c>
+      <c r="B20" s="14">
+        <v>420</v>
+      </c>
+      <c r="C20" s="14">
+        <v>60</v>
+      </c>
+      <c r="D20" s="14">
+        <v>300</v>
+      </c>
+      <c r="E20" s="14">
+        <v>120</v>
+      </c>
+      <c r="F20" s="14">
+        <v>350</v>
+      </c>
+      <c r="G20" s="14">
+        <v>7</v>
+      </c>
+      <c r="H20" s="14">
+        <v>0</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>1250</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="17"/>
+        <v>190</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="13"/>

</xml_diff>

<commit_message>
Updated on 10th September 2026
</commit_message>
<xml_diff>
--- a/12603864.xlsx
+++ b/12603864.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP 776\12603864\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D8E014D-5BA6-4DB5-A0F7-2A57A1FB962D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEAEA241-B4A9-4BA9-A459-CFA1B88C1D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="83">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -275,6 +275,15 @@
   </si>
   <si>
     <t>WENT REALLY GOOD</t>
+  </si>
+  <si>
+    <t>DAY WENT PRETTY NICE</t>
+  </si>
+  <si>
+    <t>TIRED</t>
+  </si>
+  <si>
+    <t>DAY WENT OK, JUST WASTED SOME TIME</t>
   </si>
 </sst>
 </file>
@@ -1744,48 +1753,96 @@
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+      <c r="A21" s="13">
+        <v>46273</v>
+      </c>
+      <c r="B21" s="14">
+        <v>420</v>
+      </c>
+      <c r="C21" s="14">
+        <v>60</v>
+      </c>
+      <c r="D21" s="14">
+        <v>320</v>
+      </c>
+      <c r="E21" s="14">
+        <v>60</v>
+      </c>
+      <c r="F21" s="14">
+        <v>350</v>
+      </c>
+      <c r="G21" s="14">
+        <v>7</v>
+      </c>
+      <c r="H21" s="14">
+        <v>0</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>1210</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
-      <c r="N21" s="17"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+        <v>230</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N21" s="17" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="13">
+        <v>46274</v>
+      </c>
+      <c r="B22" s="14">
+        <v>420</v>
+      </c>
+      <c r="C22" s="14">
+        <v>60</v>
+      </c>
+      <c r="D22" s="14">
+        <v>320</v>
+      </c>
+      <c r="E22" s="14">
+        <v>60</v>
+      </c>
+      <c r="F22" s="14">
+        <v>350</v>
+      </c>
+      <c r="G22" s="14">
+        <v>7</v>
+      </c>
+      <c r="H22" s="14">
+        <v>0</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>1210</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="17"/>
+        <v>230</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="13"/>

</xml_diff>

<commit_message>
Updated on 16th September
</commit_message>
<xml_diff>
--- a/12603864.xlsx
+++ b/12603864.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP 776\12603864\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEAEA241-B4A9-4BA9-A459-CFA1B88C1D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE574015-913C-455E-9B29-7527EA78A2A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -284,6 +284,27 @@
   </si>
   <si>
     <t>DAY WENT OK, JUST WASTED SOME TIME</t>
+  </si>
+  <si>
+    <t>VERY GOOD</t>
+  </si>
+  <si>
+    <t>DAY WENT GOOD, LITTLE PRODUCTIVE THAN OTHERS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DAY WENT GOOD </t>
+  </si>
+  <si>
+    <t>DAY WENT GOOD BUT WASTED SOME TIME</t>
+  </si>
+  <si>
+    <t>DAY DIDN'T WENT GOOD</t>
+  </si>
+  <si>
+    <t>DAY WENT OK BUT DIDN’T UTILISED THE TIME PROPERLY</t>
+  </si>
+  <si>
+    <t>JUST WASTED TIME A LOT</t>
   </si>
 </sst>
 </file>
@@ -1844,137 +1865,281 @@
         <v>82</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+    <row r="23" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="13">
+        <v>46275</v>
+      </c>
+      <c r="B23" s="14">
+        <v>420</v>
+      </c>
+      <c r="C23" s="14">
+        <v>60</v>
+      </c>
+      <c r="D23" s="14">
+        <v>360</v>
+      </c>
+      <c r="E23" s="14">
+        <v>60</v>
+      </c>
+      <c r="F23" s="14">
+        <v>250</v>
+      </c>
+      <c r="G23" s="14">
+        <v>5</v>
+      </c>
+      <c r="H23" s="14">
+        <v>0</v>
+      </c>
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>1150</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
-      <c r="N23" s="17"/>
+        <v>290</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N23" s="17" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="15" t="str">
+      <c r="A24" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B24" s="14">
+        <v>420</v>
+      </c>
+      <c r="C24" s="14">
+        <v>60</v>
+      </c>
+      <c r="D24" s="14">
+        <v>360</v>
+      </c>
+      <c r="E24" s="14">
+        <v>60</v>
+      </c>
+      <c r="F24" s="14">
+        <v>250</v>
+      </c>
+      <c r="G24" s="14">
+        <v>5</v>
+      </c>
+      <c r="H24" s="14">
+        <v>0</v>
+      </c>
+      <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
+        <v>1150</v>
+      </c>
+      <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="17"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A25" s="13"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="15" t="str">
+        <v>290</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N24" s="17" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="13">
+        <v>46277</v>
+      </c>
+      <c r="B25" s="14">
+        <v>420</v>
+      </c>
+      <c r="C25" s="14">
+        <v>60</v>
+      </c>
+      <c r="D25" s="14">
+        <v>480</v>
+      </c>
+      <c r="E25" s="14">
+        <v>60</v>
+      </c>
+      <c r="F25" s="14">
+        <v>0</v>
+      </c>
+      <c r="G25" s="14">
+        <v>0</v>
+      </c>
+      <c r="H25" s="14">
+        <v>0</v>
+      </c>
+      <c r="I25" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="15" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J25" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="17"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15" t="str">
+        <v>420</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="L25" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N25" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="13">
+        <v>46278</v>
+      </c>
+      <c r="B26" s="14">
+        <v>420</v>
+      </c>
+      <c r="C26" s="14">
+        <v>60</v>
+      </c>
+      <c r="D26" s="14">
+        <v>0</v>
+      </c>
+      <c r="E26" s="14">
+        <v>0</v>
+      </c>
+      <c r="F26" s="14">
+        <v>0</v>
+      </c>
+      <c r="G26" s="14">
+        <v>0</v>
+      </c>
+      <c r="H26" s="14">
+        <v>480</v>
+      </c>
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="15" t="str">
+        <v>960</v>
+      </c>
+      <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
-      <c r="N26" s="17"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="15" t="str">
+        <v>480</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="N26" s="17" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="13">
+        <v>46279</v>
+      </c>
+      <c r="B27" s="14">
+        <v>420</v>
+      </c>
+      <c r="C27" s="14">
+        <v>60</v>
+      </c>
+      <c r="D27" s="14">
+        <v>300</v>
+      </c>
+      <c r="E27" s="14">
+        <v>60</v>
+      </c>
+      <c r="F27" s="14">
+        <v>350</v>
+      </c>
+      <c r="G27" s="14">
+        <v>7</v>
+      </c>
+      <c r="H27" s="14">
+        <v>0</v>
+      </c>
+      <c r="I27" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
+        <v>1190</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="17"/>
+        <v>250</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N27" s="17" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+      <c r="A28" s="13">
+        <v>46280</v>
+      </c>
+      <c r="B28" s="14">
+        <v>420</v>
+      </c>
+      <c r="C28" s="14">
+        <v>60</v>
+      </c>
+      <c r="D28" s="14">
+        <v>0</v>
+      </c>
+      <c r="E28" s="14">
+        <v>60</v>
+      </c>
+      <c r="F28" s="14">
+        <v>350</v>
+      </c>
+      <c r="G28" s="14">
+        <v>7</v>
+      </c>
+      <c r="H28" s="14">
+        <v>120</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>1010</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="17"/>
+        <v>430</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="13"/>

</xml_diff>

<commit_message>
Updated on 17th September 2026
</commit_message>
<xml_diff>
--- a/12603864.xlsx
+++ b/12603864.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP 776\12603864\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE574015-913C-455E-9B29-7527EA78A2A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6321A468-C2F6-4411-885B-1A0D57399FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="91">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -305,6 +305,9 @@
   </si>
   <si>
     <t>JUST WASTED TIME A LOT</t>
+  </si>
+  <si>
+    <t>DID QUANTS TODAY, IT WENT GOOD</t>
   </si>
 </sst>
 </file>
@@ -2141,27 +2144,51 @@
         <v>89</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+    <row r="29" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="13">
+        <v>46281</v>
+      </c>
+      <c r="B29" s="14">
+        <v>420</v>
+      </c>
+      <c r="C29" s="14">
+        <v>60</v>
+      </c>
+      <c r="D29" s="14">
+        <v>270</v>
+      </c>
+      <c r="E29" s="14">
+        <v>0</v>
+      </c>
+      <c r="F29" s="14">
+        <v>350</v>
+      </c>
+      <c r="G29" s="14">
+        <v>7</v>
+      </c>
+      <c r="H29" s="14">
+        <v>60</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>1160</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="17"/>
+        <v>280</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N29" s="17" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="13"/>

</xml_diff>

<commit_message>
Updated on 19th September 2026
</commit_message>
<xml_diff>
--- a/12603864.xlsx
+++ b/12603864.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP 776\12603864\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6321A468-C2F6-4411-885B-1A0D57399FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F12971D-618A-473C-B36A-93B2E8AD38A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="92">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -307,7 +307,10 @@
     <t>JUST WASTED TIME A LOT</t>
   </si>
   <si>
-    <t>DID QUANTS TODAY, IT WENT GOOD</t>
+    <t>DID QUANTS TODAY</t>
+  </si>
+  <si>
+    <t>DID NOTHING TODAY</t>
   </si>
 </sst>
 </file>
@@ -2144,7 +2147,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="13">
         <v>46281</v>
       </c>
@@ -2191,48 +2194,96 @@
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15" t="str">
+      <c r="A30" s="13">
+        <v>46282</v>
+      </c>
+      <c r="B30" s="14">
+        <v>420</v>
+      </c>
+      <c r="C30" s="14">
+        <v>60</v>
+      </c>
+      <c r="D30" s="14">
+        <v>300</v>
+      </c>
+      <c r="E30" s="14">
+        <v>0</v>
+      </c>
+      <c r="F30" s="14">
+        <v>350</v>
+      </c>
+      <c r="G30" s="14">
+        <v>7</v>
+      </c>
+      <c r="H30" s="14">
+        <v>0</v>
+      </c>
+      <c r="I30" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
+        <v>1130</v>
+      </c>
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="17"/>
+        <v>310</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="13"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="15" t="str">
+      <c r="A31" s="13">
+        <v>46283</v>
+      </c>
+      <c r="B31" s="14">
+        <v>420</v>
+      </c>
+      <c r="C31" s="14">
+        <v>0</v>
+      </c>
+      <c r="D31" s="14">
+        <v>0</v>
+      </c>
+      <c r="E31" s="14">
+        <v>0</v>
+      </c>
+      <c r="F31" s="14">
+        <v>0</v>
+      </c>
+      <c r="G31" s="14">
+        <v>0</v>
+      </c>
+      <c r="H31" s="14">
+        <v>800</v>
+      </c>
+      <c r="I31" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
+        <v>1220</v>
+      </c>
+      <c r="J31" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="17"/>
+        <v>220</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N31" s="17" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="13"/>

</xml_diff>